<commit_message>
Phase 1-5 complete - UI, confidence scores, RPA, Gmail, logging
</commit_message>
<xml_diff>
--- a/invoice_records.xlsx
+++ b/invoice_records.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -504,6 +504,202 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ABC Digital Solutions Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>INV-2026-001</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>03-Jul-2026</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>64900</v>
+      </c>
+      <c r="E4" t="n">
+        <v>9900</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TechNova Solutions Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TN-2026-014</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>04-Jul-2026</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>90860</v>
+      </c>
+      <c r="E5" t="n">
+        <v>13860</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TechNova Solutions Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TN-2026-014</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>04-Jul-2026</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>90860</v>
+      </c>
+      <c r="E6" t="n">
+        <v>13860</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NextGen Software Services LLP</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>NG-2026-027</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>06-Jul-2026</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>118000</v>
+      </c>
+      <c r="E7" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TechNova Solutions Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TN-2026-014</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>04-Jul-2026</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>90860</v>
+      </c>
+      <c r="E8" t="n">
+        <v>13860</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TechNova Solutions Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TN-2026-014</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>04-Jul-2026</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>90860</v>
+      </c>
+      <c r="E9" t="n">
+        <v>13860</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TechNova Solutions Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TN-2026-014</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>04-Jul-2026</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>90860</v>
+      </c>
+      <c r="E10" t="n">
+        <v>13860</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added AI Fraud Detection system
</commit_message>
<xml_diff>
--- a/invoice_records.xlsx
+++ b/invoice_records.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -728,6 +728,34 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ABC Digital Solutions Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>INV-2026-001</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>03-Jul-2026</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>64900</v>
+      </c>
+      <c r="E12" t="n">
+        <v>9900</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Processed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>